<commit_message>
Beam characterization kinda done
</commit_message>
<xml_diff>
--- a/BeamChar/BEAM2.xlsx
+++ b/BeamChar/BEAM2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\37259\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\37259\Desktop\kool\VSC-random\BeamChar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{886AD4FD-921F-4159-BFF8-EE1ADB286219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8F505F6-A519-426E-94C7-48224143FFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Distance</t>
   </si>
@@ -75,6 +75,18 @@
   </si>
   <si>
     <t>holes</t>
+  </si>
+  <si>
+    <t>Diff Y</t>
+  </si>
+  <si>
+    <t>Diff X (ellips minor - clip X)</t>
+  </si>
+  <si>
+    <t>ellipoticity</t>
+  </si>
+  <si>
+    <t>ellipticity from clip</t>
   </si>
 </sst>
 </file>
@@ -387,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:Z17"/>
+  <dimension ref="A4:Z21"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="41.77734375" customWidth="1"/>
@@ -482,11 +494,11 @@
         <v>55.8</v>
       </c>
       <c r="C5">
-        <f t="shared" ref="C5:Z5" si="0">(C4-9)*25.4</f>
+        <f>(C4-9)*25.4</f>
         <v>101.6</v>
       </c>
       <c r="D5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="D5:Z5" si="0">(D4-9)*25.4</f>
         <v>152.39999999999998</v>
       </c>
       <c r="E5">
@@ -1536,6 +1548,426 @@
       </c>
       <c r="Z17">
         <v>5097.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18">
+        <f>B12-B14</f>
+        <v>-87.5</v>
+      </c>
+      <c r="C18">
+        <f t="shared" ref="C18:Z18" si="1">C12-C14</f>
+        <v>-108.70000000000005</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="1"/>
+        <v>-136.20000000000005</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="1"/>
+        <v>-160</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="1"/>
+        <v>-192.70000000000005</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="1"/>
+        <v>-217.20000000000005</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="1"/>
+        <v>-258.70000000000005</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="1"/>
+        <v>-285.49999999999977</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="1"/>
+        <v>-306</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="1"/>
+        <v>-323.5</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="1"/>
+        <v>-349</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="1"/>
+        <v>-372.19999999999982</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="1"/>
+        <v>-384.40000000000009</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="1"/>
+        <v>-400.30000000000018</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="1"/>
+        <v>-409.5</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="1"/>
+        <v>-444.90000000000009</v>
+      </c>
+      <c r="R18">
+        <f t="shared" si="1"/>
+        <v>-486.60000000000036</v>
+      </c>
+      <c r="S18">
+        <f t="shared" si="1"/>
+        <v>-507.89999999999964</v>
+      </c>
+      <c r="T18">
+        <f t="shared" si="1"/>
+        <v>-529.09999999999945</v>
+      </c>
+      <c r="U18">
+        <f t="shared" si="1"/>
+        <v>-546.60000000000036</v>
+      </c>
+      <c r="V18">
+        <f t="shared" si="1"/>
+        <v>-543.19999999999982</v>
+      </c>
+      <c r="W18">
+        <f t="shared" si="1"/>
+        <v>-570.59999999999945</v>
+      </c>
+      <c r="X18">
+        <f t="shared" si="1"/>
+        <v>-596.80000000000018</v>
+      </c>
+      <c r="Y18">
+        <f t="shared" si="1"/>
+        <v>-605.5</v>
+      </c>
+      <c r="Z18">
+        <f t="shared" si="1"/>
+        <v>-614.89999999999964</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19">
+        <f>+B13-B15</f>
+        <v>32.400000000000091</v>
+      </c>
+      <c r="C19">
+        <f t="shared" ref="C19:Z19" si="2">+C13-C15</f>
+        <v>63.899999999999977</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="2"/>
+        <v>78.899999999999864</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="2"/>
+        <v>88.700000000000045</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="2"/>
+        <v>93.900000000000091</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="2"/>
+        <v>101</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="2"/>
+        <v>124.39999999999986</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="2"/>
+        <v>140.89999999999964</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="2"/>
+        <v>155.69999999999982</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="2"/>
+        <v>170.40000000000009</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="2"/>
+        <v>182.5</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="2"/>
+        <v>194.29999999999973</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="2"/>
+        <v>196.09999999999991</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="2"/>
+        <v>204.90000000000009</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="2"/>
+        <v>212.59999999999991</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="2"/>
+        <v>243.09999999999991</v>
+      </c>
+      <c r="R19">
+        <f t="shared" si="2"/>
+        <v>262.70000000000027</v>
+      </c>
+      <c r="S19">
+        <f t="shared" si="2"/>
+        <v>275.59999999999991</v>
+      </c>
+      <c r="T19">
+        <f t="shared" si="2"/>
+        <v>276.5</v>
+      </c>
+      <c r="U19">
+        <f t="shared" si="2"/>
+        <v>285.30000000000018</v>
+      </c>
+      <c r="V19">
+        <f t="shared" si="2"/>
+        <v>295.69999999999982</v>
+      </c>
+      <c r="W19">
+        <f t="shared" si="2"/>
+        <v>296.30000000000018</v>
+      </c>
+      <c r="X19">
+        <f t="shared" si="2"/>
+        <v>306.60000000000036</v>
+      </c>
+      <c r="Y19">
+        <f t="shared" si="2"/>
+        <v>313.5</v>
+      </c>
+      <c r="Z19">
+        <f t="shared" si="2"/>
+        <v>310.39999999999964</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20">
+        <f>+B12/B13</f>
+        <v>0.93070362473347545</v>
+      </c>
+      <c r="C20">
+        <f t="shared" ref="C20:Z20" si="3">+C12/C13</f>
+        <v>0.91945719027628625</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="3"/>
+        <v>0.91581361067889611</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="3"/>
+        <v>0.91253973860826565</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="3"/>
+        <v>0.91079667794524766</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="3"/>
+        <v>0.91034861377985177</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="3"/>
+        <v>0.90588755651661101</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="3"/>
+        <v>0.90504636233951508</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="3"/>
+        <v>0.90582023575638515</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="3"/>
+        <v>0.90588457899716179</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="3"/>
+        <v>0.90715598925187391</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="3"/>
+        <v>0.90805621536025338</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="3"/>
+        <v>0.91010784586384841</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="3"/>
+        <v>0.91030867792661618</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="3"/>
+        <v>0.91139902074049628</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="3"/>
+        <v>0.9089821605034587</v>
+      </c>
+      <c r="R20">
+        <f t="shared" si="3"/>
+        <v>0.90782681716021629</v>
+      </c>
+      <c r="S20">
+        <f t="shared" si="3"/>
+        <v>0.9086943193340723</v>
+      </c>
+      <c r="T20">
+        <f t="shared" si="3"/>
+        <v>0.91059423363263092</v>
+      </c>
+      <c r="U20">
+        <f t="shared" si="3"/>
+        <v>0.91143417959060413</v>
+      </c>
+      <c r="V20">
+        <f t="shared" si="3"/>
+        <v>0.91314285714285715</v>
+      </c>
+      <c r="W20">
+        <f t="shared" si="3"/>
+        <v>0.91531081351189292</v>
+      </c>
+      <c r="X20">
+        <f t="shared" si="3"/>
+        <v>0.91484493664801669</v>
+      </c>
+      <c r="Y20">
+        <f t="shared" si="3"/>
+        <v>0.91436315369335586</v>
+      </c>
+      <c r="Z20">
+        <f t="shared" si="3"/>
+        <v>0.91712220384089771</v>
+      </c>
+    </row>
+    <row r="21" spans="1:26">
+      <c r="A21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21">
+        <f>B15/B14</f>
+        <v>0.92968392120934484</v>
+      </c>
+      <c r="C21">
+        <f t="shared" ref="C21:Z21" si="4">C15/C14</f>
+        <v>0.9142313184198001</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="4"/>
+        <v>0.91048226385013953</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="4"/>
+        <v>0.91396294000137768</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="4"/>
+        <v>0.91537174276834798</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="4"/>
+        <v>0.91740428708542177</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="4"/>
+        <v>0.90884871550903901</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="4"/>
+        <v>0.9078464395215271</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="4"/>
+        <v>0.90806240323925214</v>
+      </c>
+      <c r="K21">
+        <f t="shared" si="4"/>
+        <v>0.90976336804916635</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="4"/>
+        <v>0.907746672155894</v>
+      </c>
+      <c r="M21">
+        <f t="shared" si="4"/>
+        <v>0.90789515793516185</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="4"/>
+        <v>0.91302258529553104</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="4"/>
+        <v>0.91571902560757723</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="4"/>
+        <v>0.91941549371440856</v>
+      </c>
+      <c r="Q21">
+        <f t="shared" si="4"/>
+        <v>0.91421972946222374</v>
+      </c>
+      <c r="R21">
+        <f t="shared" si="4"/>
+        <v>0.90964130408668276</v>
+      </c>
+      <c r="S21">
+        <f t="shared" si="4"/>
+        <v>0.90913468152428123</v>
+      </c>
+      <c r="T21">
+        <f t="shared" si="4"/>
+        <v>0.9103473956279845</v>
+      </c>
+      <c r="U21">
+        <f t="shared" si="4"/>
+        <v>0.91171601600972318</v>
+      </c>
+      <c r="V21">
+        <f t="shared" si="4"/>
+        <v>0.91475788322498341</v>
+      </c>
+      <c r="W21">
+        <f t="shared" si="4"/>
+        <v>0.9139400765063399</v>
+      </c>
+      <c r="X21">
+        <f t="shared" si="4"/>
+        <v>0.91400560224089633</v>
+      </c>
+      <c r="Y21">
+        <f t="shared" si="4"/>
+        <v>0.91724674103672099</v>
+      </c>
+      <c r="Z21">
+        <f t="shared" si="4"/>
+        <v>0.91874300111982088</v>
       </c>
     </row>
   </sheetData>

</xml_diff>